<commit_message>
Innkeeper and Barkeep trades and conversations in Minoc.  Room mechanic for Minoc (different from Skara)
</commit_message>
<xml_diff>
--- a/spoilers/conversations.xlsx
+++ b/spoilers/conversations.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\MYDATA\_GIT_REPOS\mcu4\spoilers\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{8AABCEE6-E0E6-4BC9-BD68-16C493184F7B}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{1B1DF0D3-C086-448F-978D-5C92D672C688}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="11964" activeTab="1" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -28,7 +28,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="4711" uniqueCount="1443">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="4756" uniqueCount="1461">
   <si>
     <t>Game-Level Conversation List</t>
   </si>
@@ -4381,6 +4381,60 @@
   </si>
   <si>
     <t>Estrol: Then speak to the judge in Yew!</t>
+  </si>
+  <si>
+    <t>Rooms</t>
+  </si>
+  <si>
+    <t>3, 6, or 9 gold nuggets -- finer stays cost more.</t>
+  </si>
+  <si>
+    <t>Estro: Rooms for rent -- 3, 6, or 9 gold nuggets, finer stays cost more. See my trades.</t>
+  </si>
+  <si>
+    <t>gold-&gt;copper (3)</t>
+  </si>
+  <si>
+    <t>Estro: Here's your change -- room's ready, door shuts in 20s.</t>
+  </si>
+  <si>
+    <t>Opens room-1 door, 20s auto-checkout; if occupied, refunds 3 gold instead and declines</t>
+  </si>
+  <si>
+    <t>gold-&gt;copper (6)</t>
+  </si>
+  <si>
+    <t>Opens room-2 door, same pattern, refund 6 gold if occupied</t>
+  </si>
+  <si>
+    <t>gold-&gt;copper (9)</t>
+  </si>
+  <si>
+    <t>Opens room-3 door, same pattern, refund 9 gold if occupied</t>
+  </si>
+  <si>
+    <t>OK, room 2. Here's your change.</t>
+  </si>
+  <si>
+    <t>OK, room 1. Here's your change.</t>
+  </si>
+  <si>
+    <t>OK, room 3. Here's your change.</t>
+  </si>
+  <si>
+    <t>Butch</t>
+  </si>
+  <si>
+    <t>Barkeep</t>
+  </si>
+  <si>
+    <t>Want Food?</t>
+  </si>
+  <si>
+    <t>We've got a fine selection of goods.</t>
+  </si>
+  <si>
+    <t>Butch: We've got a fine selection of goods.</t>
   </si>
 </sst>
 </file>
@@ -37150,7 +37204,7 @@
   <sheetPr>
     <tabColor rgb="FF92D050"/>
   </sheetPr>
-  <dimension ref="A1:O495"/>
+  <dimension ref="A1:O499"/>
   <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
   <cols>
     <col min="1" max="1" width="10" customWidth="1"/>
@@ -39373,7 +39427,7 @@
       </c>
       <c r="H53" s="5"/>
       <c r="I53" s="5">
-        <f>INT((1/COUNTIF(B:B,B53))*100)</f>
+        <f t="shared" ref="I53:I91" si="0">INT((1/COUNTIF(B:B,B53))*100)</f>
         <v>16</v>
       </c>
       <c r="J53" s="5" t="s">
@@ -39417,7 +39471,7 @@
         <v>73</v>
       </c>
       <c r="I54" s="5">
-        <f>INT((1/COUNTIF(B:B,B54))*100)</f>
+        <f t="shared" si="0"/>
         <v>16</v>
       </c>
       <c r="J54" s="5" t="s">
@@ -39463,7 +39517,7 @@
         <v>77</v>
       </c>
       <c r="I55" s="5">
-        <f>INT((1/COUNTIF(B:B,B55))*100)</f>
+        <f t="shared" si="0"/>
         <v>16</v>
       </c>
       <c r="J55" s="5" t="s">
@@ -39503,7 +39557,7 @@
       </c>
       <c r="H56" s="5"/>
       <c r="I56" s="5">
-        <f>INT((1/COUNTIF(B:B,B56))*100)</f>
+        <f t="shared" si="0"/>
         <v>16</v>
       </c>
       <c r="J56" s="5" t="s">
@@ -39545,7 +39599,7 @@
       </c>
       <c r="H57" s="5"/>
       <c r="I57" s="5">
-        <f>INT((1/COUNTIF(B:B,B57))*100)</f>
+        <f t="shared" si="0"/>
         <v>16</v>
       </c>
       <c r="J57" s="5" t="s">
@@ -39586,7 +39640,7 @@
       </c>
       <c r="H58" s="5"/>
       <c r="I58" s="5">
-        <f>INT((1/COUNTIF(B:B,B58))*100)</f>
+        <f t="shared" si="0"/>
         <v>33</v>
       </c>
       <c r="J58" s="24" t="s">
@@ -39628,7 +39682,7 @@
       </c>
       <c r="H59" s="5"/>
       <c r="I59" s="5">
-        <f>INT((1/COUNTIF(B:B,B59))*100)</f>
+        <f t="shared" si="0"/>
         <v>33</v>
       </c>
       <c r="J59" s="24" t="s">
@@ -39638,7 +39692,7 @@
         <v>283</v>
       </c>
       <c r="L59" s="5" t="str">
-        <f t="shared" ref="L59:L98" si="0">B59&amp;": "&amp;K59</f>
+        <f t="shared" ref="L59:L98" si="1">B59&amp;": "&amp;K59</f>
         <v>Browning: I strive to live an honest life!</v>
       </c>
       <c r="M59" s="5"/>
@@ -39670,7 +39724,7 @@
       </c>
       <c r="H60" s="5"/>
       <c r="I60" s="5">
-        <f>INT((1/COUNTIF(B:B,B60))*100)</f>
+        <f t="shared" si="0"/>
         <v>33</v>
       </c>
       <c r="J60" s="24" t="s">
@@ -39680,7 +39734,7 @@
         <v>316</v>
       </c>
       <c r="L60" s="5" t="str">
-        <f t="shared" si="0"/>
+        <f t="shared" si="1"/>
         <v>Browning: It is rooted in Knowledge and Courage.</v>
       </c>
       <c r="M60" s="5"/>
@@ -39712,7 +39766,7 @@
       </c>
       <c r="H61" s="5"/>
       <c r="I61" s="5">
-        <f>INT((1/COUNTIF(B:B,B61))*100)</f>
+        <f t="shared" si="0"/>
         <v>33</v>
       </c>
       <c r="J61" s="25" t="s">
@@ -39722,7 +39776,7 @@
         <v>344</v>
       </c>
       <c r="L61" s="5" t="str">
-        <f t="shared" si="0"/>
+        <f t="shared" si="1"/>
         <v>Calabrini: Yes several types of potions are sold here!</v>
       </c>
       <c r="M61" s="5"/>
@@ -39754,7 +39808,7 @@
       </c>
       <c r="H62" s="5"/>
       <c r="I62" s="5">
-        <f>INT((1/COUNTIF(B:B,B62))*100)</f>
+        <f t="shared" si="0"/>
         <v>33</v>
       </c>
       <c r="J62" s="24" t="s">
@@ -39764,7 +39818,7 @@
         <v>348</v>
       </c>
       <c r="L62" s="5" t="str">
-        <f t="shared" si="0"/>
+        <f t="shared" si="1"/>
         <v>Calabrini: The housekeeper at the inn is very chatty.</v>
       </c>
       <c r="M62" s="5"/>
@@ -39796,7 +39850,7 @@
       </c>
       <c r="H63" s="5"/>
       <c r="I63" s="5">
-        <f>INT((1/COUNTIF(B:B,B63))*100)</f>
+        <f t="shared" si="0"/>
         <v>33</v>
       </c>
       <c r="J63" s="24" t="s">
@@ -39806,7 +39860,7 @@
         <v>345</v>
       </c>
       <c r="L63" s="5" t="str">
-        <f t="shared" si="0"/>
+        <f t="shared" si="1"/>
         <v>Calabrini: I bear greetings from the HONEST town of Moonglow.</v>
       </c>
       <c r="M63" s="5"/>
@@ -39838,7 +39892,7 @@
       </c>
       <c r="H64" s="5"/>
       <c r="I64" s="5">
-        <f>INT((1/COUNTIF(B:B,B64))*100)</f>
+        <f t="shared" si="0"/>
         <v>20</v>
       </c>
       <c r="J64" s="25" t="s">
@@ -39848,7 +39902,7 @@
         <v>284</v>
       </c>
       <c r="L64" s="5" t="str">
-        <f t="shared" si="0"/>
+        <f t="shared" si="1"/>
         <v>Christen: Honest friends are few!</v>
       </c>
       <c r="M64" s="5"/>
@@ -39880,7 +39934,7 @@
       </c>
       <c r="H65" s="5"/>
       <c r="I65" s="5">
-        <f>INT((1/COUNTIF(B:B,B65))*100)</f>
+        <f t="shared" si="0"/>
         <v>20</v>
       </c>
       <c r="J65" s="24" t="s">
@@ -39890,7 +39944,7 @@
         <v>319</v>
       </c>
       <c r="L65" s="5" t="str">
-        <f t="shared" si="0"/>
+        <f t="shared" si="1"/>
         <v>Christen: Imma feeling gooood!</v>
       </c>
       <c r="M65" s="5"/>
@@ -39922,7 +39976,7 @@
       </c>
       <c r="H66" s="5"/>
       <c r="I66" s="5">
-        <f>INT((1/COUNTIF(B:B,B66))*100)</f>
+        <f t="shared" si="0"/>
         <v>20</v>
       </c>
       <c r="J66" s="24" t="s">
@@ -39932,7 +39986,7 @@
         <v>285</v>
       </c>
       <c r="L66" s="5" t="str">
-        <f t="shared" si="0"/>
+        <f t="shared" si="1"/>
         <v>Christen: My friend William knows where the rune of honesty is.</v>
       </c>
       <c r="M66" s="5"/>
@@ -39964,7 +40018,7 @@
       </c>
       <c r="H67" s="5"/>
       <c r="I67" s="5">
-        <f>INT((1/COUNTIF(B:B,B67))*100)</f>
+        <f t="shared" si="0"/>
         <v>20</v>
       </c>
       <c r="J67" s="24" t="s">
@@ -39974,7 +40028,7 @@
         <v>349</v>
       </c>
       <c r="L67" s="26" t="str">
-        <f t="shared" si="0"/>
+        <f t="shared" si="1"/>
         <v>Christen: Hey, don't open Rebelias' personal chests. That's not honest!</v>
       </c>
       <c r="M67" s="5"/>
@@ -40006,7 +40060,7 @@
       </c>
       <c r="H68" s="5"/>
       <c r="I68" s="5">
-        <f>INT((1/COUNTIF(B:B,B68))*100)</f>
+        <f t="shared" si="0"/>
         <v>20</v>
       </c>
       <c r="J68" s="24" t="s">
@@ -40016,7 +40070,7 @@
         <v>286</v>
       </c>
       <c r="L68" s="5" t="str">
-        <f t="shared" si="0"/>
+        <f t="shared" si="1"/>
         <v>Christen: The housekeeping nitwit.</v>
       </c>
       <c r="M68" s="5"/>
@@ -40048,7 +40102,7 @@
       </c>
       <c r="H69" s="5"/>
       <c r="I69" s="5">
-        <f>INT((1/COUNTIF(B:B,B69))*100)</f>
+        <f t="shared" si="0"/>
         <v>33</v>
       </c>
       <c r="J69" s="24" t="s">
@@ -40058,7 +40112,7 @@
         <v>287</v>
       </c>
       <c r="L69" s="5" t="str">
-        <f t="shared" si="0"/>
+        <f t="shared" si="1"/>
         <v>Cromwell: A few honest men are better than numbers!</v>
       </c>
       <c r="M69" s="5"/>
@@ -40090,7 +40144,7 @@
       </c>
       <c r="H70" s="5"/>
       <c r="I70" s="5">
-        <f>INT((1/COUNTIF(B:B,B70))*100)</f>
+        <f t="shared" si="0"/>
         <v>33</v>
       </c>
       <c r="J70" s="24" t="s">
@@ -40100,7 +40154,7 @@
         <v>288</v>
       </c>
       <c r="L70" s="5" t="str">
-        <f t="shared" si="0"/>
+        <f t="shared" si="1"/>
         <v>Cromwell: I speak of the virtues of honesty!</v>
       </c>
       <c r="M70" s="5"/>
@@ -40132,7 +40186,7 @@
       </c>
       <c r="H71" s="5"/>
       <c r="I71" s="5">
-        <f>INT((1/COUNTIF(B:B,B71))*100)</f>
+        <f t="shared" si="0"/>
         <v>33</v>
       </c>
       <c r="J71" s="24" t="s">
@@ -40142,7 +40196,7 @@
         <v>289</v>
       </c>
       <c r="L71" s="5" t="str">
-        <f t="shared" si="0"/>
+        <f t="shared" si="1"/>
         <v>Cromwell: The mantra for Honesty is ’AHM’.</v>
       </c>
       <c r="M71" s="5"/>
@@ -40174,7 +40228,7 @@
       </c>
       <c r="H72" s="5"/>
       <c r="I72" s="5">
-        <f>INT((1/COUNTIF(B:B,B72))*100)</f>
+        <f t="shared" si="0"/>
         <v>33</v>
       </c>
       <c r="J72" s="24" t="s">
@@ -40184,7 +40238,7 @@
         <v>342</v>
       </c>
       <c r="L72" s="5" t="str">
-        <f t="shared" si="0"/>
+        <f t="shared" si="1"/>
         <v>Mariah: Yes, I hope to go on a great quest, one day!</v>
       </c>
       <c r="M72" s="5"/>
@@ -40216,7 +40270,7 @@
       </c>
       <c r="H73" s="5"/>
       <c r="I73" s="5">
-        <f>INT((1/COUNTIF(B:B,B73))*100)</f>
+        <f t="shared" si="0"/>
         <v>33</v>
       </c>
       <c r="J73" s="24" t="s">
@@ -40226,7 +40280,7 @@
         <v>341</v>
       </c>
       <c r="L73" s="5" t="str">
-        <f t="shared" si="0"/>
+        <f t="shared" si="1"/>
         <v>Mariah: I tend to the pond fish. It's honest work.</v>
       </c>
       <c r="M73" s="5"/>
@@ -40258,7 +40312,7 @@
       </c>
       <c r="H74" s="5"/>
       <c r="I74" s="5">
-        <f>INT((1/COUNTIF(B:B,B74))*100)</f>
+        <f t="shared" si="0"/>
         <v>33</v>
       </c>
       <c r="J74" s="24" t="s">
@@ -40268,7 +40322,7 @@
         <v>290</v>
       </c>
       <c r="L74" s="5" t="str">
-        <f t="shared" si="0"/>
+        <f t="shared" si="1"/>
         <v>Mariah: The quest of the avatar is noble indeed!</v>
       </c>
       <c r="M74" s="5"/>
@@ -40300,7 +40354,7 @@
       </c>
       <c r="H75" s="5"/>
       <c r="I75" s="5">
-        <f>INT((1/COUNTIF(B:B,B75))*100)</f>
+        <f t="shared" si="0"/>
         <v>33</v>
       </c>
       <c r="J75" s="24" t="s">
@@ -40310,7 +40364,7 @@
         <v>317</v>
       </c>
       <c r="L75" s="5" t="str">
-        <f t="shared" si="0"/>
+        <f t="shared" si="1"/>
         <v>Patric the Humble Shepherd: Humility is not derived from any of the four principles.</v>
       </c>
       <c r="M75" s="5"/>
@@ -40342,7 +40396,7 @@
       </c>
       <c r="H76" s="5"/>
       <c r="I76" s="5">
-        <f>INT((1/COUNTIF(B:B,B76))*100)</f>
+        <f t="shared" si="0"/>
         <v>33</v>
       </c>
       <c r="J76" s="24" t="s">
@@ -40352,7 +40406,7 @@
         <v>318</v>
       </c>
       <c r="L76" s="5" t="str">
-        <f t="shared" si="0"/>
+        <f t="shared" si="1"/>
         <v>Patric the Humble Shepherd: Humility is to act while remaining humble.</v>
       </c>
       <c r="M76" s="5"/>
@@ -40384,7 +40438,7 @@
       </c>
       <c r="H77" s="5"/>
       <c r="I77" s="5">
-        <f>INT((1/COUNTIF(B:B,B77))*100)</f>
+        <f t="shared" si="0"/>
         <v>33</v>
       </c>
       <c r="J77" s="24" t="s">
@@ -40394,7 +40448,7 @@
         <v>291</v>
       </c>
       <c r="L77" s="5" t="str">
-        <f t="shared" si="0"/>
+        <f t="shared" si="1"/>
         <v>Patric the Humble Shepherd: I am a meek shepherd.</v>
       </c>
       <c r="M77" s="5"/>
@@ -40426,7 +40480,7 @@
       </c>
       <c r="H78" s="5"/>
       <c r="I78" s="5">
-        <f>INT((1/COUNTIF(B:B,B78))*100)</f>
+        <f t="shared" si="0"/>
         <v>33</v>
       </c>
       <c r="J78" s="24" t="s">
@@ -40436,7 +40490,7 @@
         <v>292</v>
       </c>
       <c r="L78" s="5" t="str">
-        <f t="shared" si="0"/>
+        <f t="shared" si="1"/>
         <v>Rebelias: Evil still exists in our hearts and souls!</v>
       </c>
       <c r="M78" s="5"/>
@@ -40468,7 +40522,7 @@
       </c>
       <c r="H79" s="5"/>
       <c r="I79" s="5">
-        <f>INT((1/COUNTIF(B:B,B79))*100)</f>
+        <f t="shared" si="0"/>
         <v>33</v>
       </c>
       <c r="J79" s="24" t="s">
@@ -40478,7 +40532,7 @@
         <v>328</v>
       </c>
       <c r="L79" s="5" t="str">
-        <f t="shared" si="0"/>
+        <f t="shared" si="1"/>
         <v>Rebelias: Speak the truth always and shame evil forces!</v>
       </c>
       <c r="M79" s="5"/>
@@ -40510,7 +40564,7 @@
       </c>
       <c r="H80" s="5"/>
       <c r="I80" s="5">
-        <f>INT((1/COUNTIF(B:B,B80))*100)</f>
+        <f t="shared" si="0"/>
         <v>33</v>
       </c>
       <c r="J80" s="24" t="s">
@@ -40520,7 +40574,7 @@
         <v>293</v>
       </c>
       <c r="L80" s="5" t="str">
-        <f t="shared" si="0"/>
+        <f t="shared" si="1"/>
         <v>Rebelias: I live an honest life as a mystic wizard.</v>
       </c>
       <c r="M80" s="5"/>
@@ -40552,7 +40606,7 @@
       </c>
       <c r="H81" s="5"/>
       <c r="I81" s="5">
-        <f>INT((1/COUNTIF(B:B,B81))*100)</f>
+        <f t="shared" si="0"/>
         <v>100</v>
       </c>
       <c r="J81" s="29" t="s">
@@ -40562,7 +40616,7 @@
         <v>294</v>
       </c>
       <c r="L81" s="5" t="str">
-        <f t="shared" si="0"/>
+        <f t="shared" si="1"/>
         <v>Scatu: I am the Proprietor of Inn</v>
       </c>
       <c r="M81" s="5"/>
@@ -40594,7 +40648,7 @@
       </c>
       <c r="H82" s="5"/>
       <c r="I82" s="5">
-        <f>INT((1/COUNTIF(B:B,B82))*100)</f>
+        <f t="shared" si="0"/>
         <v>20</v>
       </c>
       <c r="J82" s="24" t="s">
@@ -40604,7 +40658,7 @@
         <v>295</v>
       </c>
       <c r="L82" s="5" t="str">
-        <f t="shared" si="0"/>
+        <f t="shared" si="1"/>
         <v>Shakespeare: Corruption wins not more than honesty!</v>
       </c>
       <c r="M82" s="5"/>
@@ -40636,7 +40690,7 @@
       </c>
       <c r="H83" s="5"/>
       <c r="I83" s="5">
-        <f>INT((1/COUNTIF(B:B,B83))*100)</f>
+        <f t="shared" si="0"/>
         <v>20</v>
       </c>
       <c r="J83" s="24" t="s">
@@ -40646,7 +40700,7 @@
         <v>296</v>
       </c>
       <c r="L83" s="5" t="str">
-        <f t="shared" si="0"/>
+        <f t="shared" si="1"/>
         <v>Shakespeare: Remember, there is no terror in threats for I am strong in honesty!</v>
       </c>
       <c r="M83" s="5"/>
@@ -40678,7 +40732,7 @@
       </c>
       <c r="H84" s="5"/>
       <c r="I84" s="5">
-        <f>INT((1/COUNTIF(B:B,B84))*100)</f>
+        <f t="shared" si="0"/>
         <v>20</v>
       </c>
       <c r="J84" s="24" t="s">
@@ -40688,7 +40742,7 @@
         <v>297</v>
       </c>
       <c r="L84" s="5" t="str">
-        <f t="shared" si="0"/>
+        <f t="shared" si="1"/>
         <v>Shakespeare: I create tales of honesty.</v>
       </c>
       <c r="M84" s="5"/>
@@ -40720,7 +40774,7 @@
       </c>
       <c r="H85" s="5"/>
       <c r="I85" s="5">
-        <f>INT((1/COUNTIF(B:B,B85))*100)</f>
+        <f t="shared" si="0"/>
         <v>20</v>
       </c>
       <c r="J85" s="29" t="s">
@@ -40730,7 +40784,7 @@
         <v>298</v>
       </c>
       <c r="L85" s="5" t="str">
-        <f t="shared" si="0"/>
+        <f t="shared" si="1"/>
         <v>Shakespeare: A wise wizard.</v>
       </c>
       <c r="M85" s="5"/>
@@ -40762,7 +40816,7 @@
       </c>
       <c r="H86" s="5"/>
       <c r="I86" s="5">
-        <f>INT((1/COUNTIF(B:B,B86))*100)</f>
+        <f t="shared" si="0"/>
         <v>20</v>
       </c>
       <c r="J86" s="24" t="s">
@@ -40772,7 +40826,7 @@
         <v>274</v>
       </c>
       <c r="L86" s="5" t="str">
-        <f t="shared" si="0"/>
+        <f t="shared" si="1"/>
         <v>Shakespeare: Shakespeare</v>
       </c>
       <c r="M86" s="5"/>
@@ -40804,7 +40858,7 @@
       </c>
       <c r="H87" s="5"/>
       <c r="I87" s="5">
-        <f>INT((1/COUNTIF(B:B,B87))*100)</f>
+        <f t="shared" si="0"/>
         <v>20</v>
       </c>
       <c r="J87" s="24" t="s">
@@ -40814,7 +40868,7 @@
         <v>299</v>
       </c>
       <c r="L87" s="5" t="str">
-        <f t="shared" si="0"/>
+        <f t="shared" si="1"/>
         <v>Shazom: I will soon die.</v>
       </c>
       <c r="M87" s="5"/>
@@ -40846,7 +40900,7 @@
       </c>
       <c r="H88" s="5"/>
       <c r="I88" s="5">
-        <f>INT((1/COUNTIF(B:B,B88))*100)</f>
+        <f t="shared" si="0"/>
         <v>20</v>
       </c>
       <c r="J88" s="24" t="s">
@@ -40856,7 +40910,7 @@
         <v>300</v>
       </c>
       <c r="L88" s="5" t="str">
-        <f t="shared" si="0"/>
+        <f t="shared" si="1"/>
         <v>Shazom: I am apprentice to the great wizard Nigel!</v>
       </c>
       <c r="M88" s="5"/>
@@ -40888,7 +40942,7 @@
       </c>
       <c r="H89" s="5"/>
       <c r="I89" s="5">
-        <f>INT((1/COUNTIF(B:B,B89))*100)</f>
+        <f t="shared" si="0"/>
         <v>20</v>
       </c>
       <c r="J89" s="29" t="s">
@@ -40898,7 +40952,7 @@
         <v>301</v>
       </c>
       <c r="L89" s="5" t="str">
-        <f t="shared" si="0"/>
+        <f t="shared" si="1"/>
         <v>Shazom: A dying young wizard.</v>
       </c>
       <c r="M89" s="5"/>
@@ -40930,7 +40984,7 @@
       </c>
       <c r="H90" s="5"/>
       <c r="I90" s="5">
-        <f>INT((1/COUNTIF(B:B,B90))*100)</f>
+        <f t="shared" si="0"/>
         <v>20</v>
       </c>
       <c r="J90" s="24" t="s">
@@ -40940,7 +40994,7 @@
         <v>275</v>
       </c>
       <c r="L90" s="5" t="str">
-        <f t="shared" si="0"/>
+        <f t="shared" si="1"/>
         <v>Shazom: Shazom</v>
       </c>
       <c r="M90" s="5"/>
@@ -40972,7 +41026,7 @@
       </c>
       <c r="H91" s="5"/>
       <c r="I91" s="5">
-        <f>INT((1/COUNTIF(B:B,B91))*100)</f>
+        <f t="shared" si="0"/>
         <v>20</v>
       </c>
       <c r="J91" s="24" t="s">
@@ -40982,7 +41036,7 @@
         <v>302</v>
       </c>
       <c r="L91" s="5" t="str">
-        <f t="shared" si="0"/>
+        <f t="shared" si="1"/>
         <v>Shazom: I will soon need to use the spell he calls ’recall’.</v>
       </c>
       <c r="M91" s="5"/>
@@ -41023,7 +41077,7 @@
         <v>303</v>
       </c>
       <c r="L92" s="5" t="str">
-        <f t="shared" si="0"/>
+        <f t="shared" si="1"/>
         <v>William: Pretty good.</v>
       </c>
       <c r="M92" s="5"/>
@@ -41064,7 +41118,7 @@
         <v>304</v>
       </c>
       <c r="L93" s="5" t="str">
-        <f t="shared" si="0"/>
+        <f t="shared" si="1"/>
         <v>William: A Nitwit eating a sandwich.</v>
       </c>
       <c r="M93" s="5"/>
@@ -41105,7 +41159,7 @@
         <v>305</v>
       </c>
       <c r="L94" s="5" t="str">
-        <f t="shared" si="0"/>
+        <f t="shared" si="1"/>
         <v>William: Search for the rune of honesty near Mariah’s gold chest!</v>
       </c>
       <c r="M94" s="5"/>
@@ -41146,7 +41200,7 @@
         <v>306</v>
       </c>
       <c r="L95" s="5" t="str">
-        <f t="shared" si="0"/>
+        <f t="shared" si="1"/>
         <v>William: It’s a peanut butter and grape jelly on lightly toasted bread!</v>
       </c>
       <c r="M95" s="5"/>
@@ -41188,7 +41242,7 @@
         <v>307</v>
       </c>
       <c r="L96" s="5" t="str">
-        <f t="shared" si="0"/>
+        <f t="shared" si="1"/>
         <v>Shaman: I am the Proprietor of Sage Deli, here.</v>
       </c>
       <c r="M96" s="5"/>
@@ -41230,7 +41284,7 @@
         <v>308</v>
       </c>
       <c r="L97" s="5" t="str">
-        <f t="shared" si="0"/>
+        <f t="shared" si="1"/>
         <v>Harmony: I am the Proprietor of The Healer shoppe.</v>
       </c>
       <c r="M97" s="5"/>
@@ -41272,7 +41326,7 @@
         <v>309</v>
       </c>
       <c r="L98" s="5" t="str">
-        <f t="shared" si="0"/>
+        <f t="shared" si="1"/>
         <v>Margot: I am the Propriety of Magical Herbs</v>
       </c>
       <c r="M98" s="5"/>
@@ -42951,7 +43005,7 @@
         <v>447</v>
       </c>
       <c r="L140" s="5" t="str">
-        <f t="shared" ref="L140:L142" si="1">B140&amp;": "&amp;K140</f>
+        <f t="shared" ref="L140:L142" si="2">B140&amp;": "&amp;K140</f>
         <v>Jumar: I am the Proprietor of Duelling Armour.</v>
       </c>
       <c r="M140" s="5"/>
@@ -42991,7 +43045,7 @@
         <v>449</v>
       </c>
       <c r="L141" s="5" t="str">
-        <f t="shared" si="1"/>
+        <f t="shared" si="2"/>
         <v>Terran: I am the Proprietor of The Keg Tap.</v>
       </c>
       <c r="M141" s="5"/>
@@ -43031,7 +43085,7 @@
         <v>448</v>
       </c>
       <c r="L142" s="5" t="str">
-        <f t="shared" si="1"/>
+        <f t="shared" si="2"/>
         <v>Zajac: I am the Proprietor of the Honorable Inn.</v>
       </c>
       <c r="M142" s="5"/>
@@ -45909,7 +45963,7 @@
         <v>740</v>
       </c>
       <c r="L214" s="46" t="str">
-        <f t="shared" ref="L214:L215" si="2">B214&amp;": "&amp;K214</f>
+        <f t="shared" ref="L214:L215" si="3">B214&amp;": "&amp;K214</f>
         <v>Faultless: Not good. Pride is a grave sin!</v>
       </c>
       <c r="M214" s="43"/>
@@ -45951,7 +46005,7 @@
         <v>741</v>
       </c>
       <c r="L215" s="46" t="str">
-        <f t="shared" si="2"/>
+        <f t="shared" si="3"/>
         <v>Faultless: Good. Pride is evil's favorite sin!</v>
       </c>
       <c r="M215" s="43"/>
@@ -46071,7 +46125,7 @@
         <v>756</v>
       </c>
       <c r="L218" s="46" t="str">
-        <f t="shared" ref="L218" si="3">B218&amp;": "&amp;K218</f>
+        <f t="shared" ref="L218" si="4">B218&amp;": "&amp;K218</f>
         <v>Heywood: I haunt eternally.</v>
       </c>
       <c r="M218" s="43"/>
@@ -46273,7 +46327,7 @@
         <v>758</v>
       </c>
       <c r="L223" s="46" t="str">
-        <f t="shared" ref="L223:L224" si="4">B223&amp;": "&amp;K223</f>
+        <f t="shared" ref="L223:L224" si="5">B223&amp;": "&amp;K223</f>
         <v>Katrina: I practice humility by meditating here.</v>
       </c>
       <c r="M223" s="43"/>
@@ -46313,7 +46367,7 @@
         <v>759</v>
       </c>
       <c r="L224" s="46" t="str">
-        <f t="shared" si="4"/>
+        <f t="shared" si="5"/>
         <v>Katrina: She looks like a worn-out survivor.</v>
       </c>
       <c r="M224" s="43"/>
@@ -46472,7 +46526,7 @@
         <v>743</v>
       </c>
       <c r="L228" s="46" t="str">
-        <f t="shared" ref="L228:L229" si="5">B228&amp;": "&amp;K228</f>
+        <f t="shared" ref="L228:L229" si="6">B228&amp;": "&amp;K228</f>
         <v>Katrina: Undo that or your efforts are meaningless.</v>
       </c>
       <c r="M228" s="43"/>
@@ -46514,7 +46568,7 @@
         <v>1308</v>
       </c>
       <c r="L229" s="46" t="str">
-        <f t="shared" si="5"/>
+        <f t="shared" si="6"/>
         <v>Katrina: The rune of Humility is in the Lycaeum.  Ignore temptations.</v>
       </c>
       <c r="M229" s="43"/>
@@ -46911,7 +46965,7 @@
         <v>744</v>
       </c>
       <c r="L239" s="46" t="str">
-        <f t="shared" ref="L239:L240" si="6">B239&amp;": "&amp;K239</f>
+        <f t="shared" ref="L239:L240" si="7">B239&amp;": "&amp;K239</f>
         <v>Virtuebane: Good! Welcome to Hell.</v>
       </c>
       <c r="M239" s="43"/>
@@ -46953,7 +47007,7 @@
         <v>753</v>
       </c>
       <c r="L240" s="46" t="str">
-        <f t="shared" si="6"/>
+        <f t="shared" si="7"/>
         <v>Virtuebane: Ah, well.  Sinners are the best winnersss…</v>
       </c>
       <c r="M240" s="43"/>
@@ -56771,11 +56825,198 @@
       </c>
     </row>
     <row r="495" spans="1:15" x14ac:dyDescent="0.3">
-      <c r="B495" s="48"/>
+      <c r="A495" t="s">
+        <v>510</v>
+      </c>
+      <c r="B495" s="48" t="s">
+        <v>533</v>
+      </c>
+      <c r="C495" t="s">
+        <v>250</v>
+      </c>
+      <c r="D495" t="s">
+        <v>61</v>
+      </c>
+      <c r="E495" t="s">
+        <v>154</v>
+      </c>
+      <c r="F495" s="16">
+        <v>-1</v>
+      </c>
+      <c r="G495" t="s">
+        <v>81</v>
+      </c>
+      <c r="J495" t="s">
+        <v>1443</v>
+      </c>
+      <c r="K495" t="s">
+        <v>1444</v>
+      </c>
+      <c r="L495" t="s">
+        <v>1445</v>
+      </c>
+      <c r="M495">
+        <v>0</v>
+      </c>
+      <c r="N495">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="496" spans="1:15" x14ac:dyDescent="0.3">
+      <c r="A496" t="s">
+        <v>510</v>
+      </c>
+      <c r="B496" t="s">
+        <v>533</v>
+      </c>
+      <c r="C496" t="s">
+        <v>250</v>
+      </c>
+      <c r="D496" t="s">
+        <v>79</v>
+      </c>
+      <c r="E496" t="s">
+        <v>1446</v>
+      </c>
+      <c r="F496" s="16">
+        <v>-1</v>
+      </c>
+      <c r="G496" t="s">
+        <v>81</v>
+      </c>
+      <c r="K496" t="s">
+        <v>1454</v>
+      </c>
+      <c r="L496" t="s">
+        <v>1447</v>
+      </c>
+      <c r="M496">
+        <v>10</v>
+      </c>
+      <c r="N496">
+        <v>0</v>
+      </c>
+      <c r="O496" t="s">
+        <v>1448</v>
+      </c>
+    </row>
+    <row r="497" spans="1:15" x14ac:dyDescent="0.3">
+      <c r="A497" t="s">
+        <v>510</v>
+      </c>
+      <c r="B497" t="s">
+        <v>533</v>
+      </c>
+      <c r="C497" t="s">
+        <v>250</v>
+      </c>
+      <c r="D497" t="s">
+        <v>79</v>
+      </c>
+      <c r="E497" t="s">
+        <v>1449</v>
+      </c>
+      <c r="F497" s="16">
+        <v>-1</v>
+      </c>
+      <c r="G497" t="s">
+        <v>81</v>
+      </c>
+      <c r="K497" t="s">
+        <v>1453</v>
+      </c>
+      <c r="L497" t="s">
+        <v>1447</v>
+      </c>
+      <c r="M497">
+        <v>10</v>
+      </c>
+      <c r="N497">
+        <v>0</v>
+      </c>
+      <c r="O497" t="s">
+        <v>1450</v>
+      </c>
+    </row>
+    <row r="498" spans="1:15" x14ac:dyDescent="0.3">
+      <c r="A498" t="s">
+        <v>510</v>
+      </c>
+      <c r="B498" t="s">
+        <v>533</v>
+      </c>
+      <c r="C498" t="s">
+        <v>250</v>
+      </c>
+      <c r="D498" t="s">
+        <v>79</v>
+      </c>
+      <c r="E498" t="s">
+        <v>1451</v>
+      </c>
+      <c r="F498" s="16">
+        <v>-1</v>
+      </c>
+      <c r="G498" t="s">
+        <v>81</v>
+      </c>
+      <c r="K498" t="s">
+        <v>1455</v>
+      </c>
+      <c r="L498" t="s">
+        <v>1447</v>
+      </c>
+      <c r="M498">
+        <v>10</v>
+      </c>
+      <c r="N498">
+        <v>0</v>
+      </c>
+      <c r="O498" t="s">
+        <v>1452</v>
+      </c>
+    </row>
+    <row r="499" spans="1:15" x14ac:dyDescent="0.3">
+      <c r="A499" t="s">
+        <v>510</v>
+      </c>
+      <c r="B499" s="48" t="s">
+        <v>1456</v>
+      </c>
+      <c r="C499" t="s">
+        <v>1457</v>
+      </c>
+      <c r="D499" t="s">
+        <v>61</v>
+      </c>
+      <c r="E499" t="s">
+        <v>154</v>
+      </c>
+      <c r="F499" s="16">
+        <v>-1</v>
+      </c>
+      <c r="G499" t="s">
+        <v>81</v>
+      </c>
+      <c r="J499" t="s">
+        <v>1458</v>
+      </c>
+      <c r="K499" t="s">
+        <v>1459</v>
+      </c>
+      <c r="L499" t="s">
+        <v>1460</v>
+      </c>
+      <c r="M499">
+        <v>0</v>
+      </c>
+      <c r="N499">
+        <v>0</v>
+      </c>
     </row>
   </sheetData>
   <autoFilter ref="A1:O494" xr:uid="{00000000-0001-0000-0100-000000000000}"/>
-  <conditionalFormatting sqref="K1:K105 K110:K111 K113:K142 K284:K319 K321:K328 K329:L330 K331:K335 K337 K339 K341:K1048576 K144:K282">
+  <conditionalFormatting sqref="K1:K105 K110:K111 K113:K142 K144:K282 K284:K319 K321:K328 K329:L330 K331:K335 K337 K339 L496:L498 K341:K1048576">
     <cfRule type="expression" dxfId="20" priority="48">
       <formula>"&gt;len(20)"</formula>
     </cfRule>

</xml_diff>